<commit_message>
MO Data description fix
</commit_message>
<xml_diff>
--- a/data/cv_entries.xlsx
+++ b/data/cv_entries.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimwright/Desktop/Resume/wright_cv/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3A17A1D-7462-0143-A9C7-9C89C53AC1F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D25A1044-A2C5-9F4E-9F89-1F0D2ACF20B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16180" xr2:uid="{C4D43CE4-6AA2-144D-A346-CE8B2E756935}"/>
   </bookViews>
@@ -342,9 +342,6 @@
     <t>Leads the WYBILT project, a series of comprehensive literacy state development grants in 25 Wyoming school districts. Responsible for consultation with the Wyoming Department of Education, overseeing data collection, analysis, and communication of findings.</t>
   </si>
   <si>
-    <t>Responsible for data wrangling and analysis of district state assessment and interim assessments to compare proficiency ratings between the type of assessment. A primary responsibility has been the development of a dashboard to communicate test results and effect size comparisons.</t>
-  </si>
-  <si>
     <t xml:space="preserve">project </t>
   </si>
   <si>
@@ -515,6 +512,9 @@
   </si>
   <si>
     <t>Developed dashboard to display results from First 5 Kern Fatherhood Initiative Survey.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Responsible for data wrangling and analysis of district state assessment and interim assessments to compare proficiency ratings between the type of assessment. </t>
   </si>
 </sst>
 </file>
@@ -993,13 +993,13 @@
         <v>15</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>137</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="409.5" x14ac:dyDescent="0.2">
@@ -1013,13 +1013,13 @@
         <v>2026</v>
       </c>
       <c r="D7" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="170" x14ac:dyDescent="0.2">
@@ -1033,13 +1033,13 @@
         <v>2025</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="F8" s="1" t="s">
         <v>111</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="187" x14ac:dyDescent="0.2">
@@ -1059,7 +1059,7 @@
         <v>73</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="170" x14ac:dyDescent="0.2">
@@ -1099,7 +1099,7 @@
         <v>73</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="102" x14ac:dyDescent="0.2">
@@ -1649,16 +1649,16 @@
         <v>15</v>
       </c>
       <c r="D43" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="F43" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="E43" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="F43" s="1" t="s">
-        <v>118</v>
-      </c>
       <c r="I43" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="44" spans="1:9" ht="238" x14ac:dyDescent="0.2">
@@ -1672,16 +1672,16 @@
         <v>15</v>
       </c>
       <c r="D44" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="F44" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="E44" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>140</v>
-      </c>
       <c r="I44" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="45" spans="1:9" ht="187" x14ac:dyDescent="0.2">
@@ -1695,13 +1695,13 @@
         <v>2024</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E45" s="1" t="s">
         <v>73</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="I45" s="1" t="s">
         <v>95</v>
@@ -1730,7 +1730,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="255" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:9" ht="136" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
         <v>86</v>
       </c>
@@ -1747,7 +1747,7 @@
         <v>73</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>102</v>
+        <v>159</v>
       </c>
       <c r="I47" s="1" t="s">
         <v>96</v>
@@ -1764,7 +1764,7 @@
         <v>2024</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E48" s="1" t="s">
         <v>73</v>
@@ -1816,7 +1816,7 @@
         <v>73</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I50" s="1" t="s">
         <v>99</v>
@@ -1824,7 +1824,7 @@
     </row>
     <row r="51" spans="1:9" ht="187" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B51" s="1">
         <v>2022</v>
@@ -1833,13 +1833,13 @@
         <v>2023</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>73</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I51" s="1" t="s">
         <v>96</v>
@@ -1893,7 +1893,7 @@
     </row>
     <row r="54" spans="1:9" ht="68" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B54" s="1">
         <v>2026</v>
@@ -1902,21 +1902,21 @@
         <v>2026</v>
       </c>
       <c r="D54" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="F54" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="E54" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="F54" s="1" t="s">
-        <v>159</v>
-      </c>
       <c r="G54" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="55" spans="1:9" ht="68" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B55" s="1">
         <v>2026</v>
@@ -1925,21 +1925,21 @@
         <v>2026</v>
       </c>
       <c r="D55" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="F55" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="E55" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="F55" s="1" t="s">
+      <c r="G55" s="1" t="s">
         <v>155</v>
-      </c>
-      <c r="G55" s="1" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="56" spans="1:9" ht="119" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B56" s="1">
         <v>2026</v>
@@ -1948,21 +1948,21 @@
         <v>2026</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="57" spans="1:9" ht="68" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B57" s="1">
         <v>2026</v>
@@ -1971,21 +1971,21 @@
         <v>2026</v>
       </c>
       <c r="D57" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="F57" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="E57" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="F57" s="1" t="s">
-        <v>150</v>
-      </c>
       <c r="G57" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="58" spans="1:9" ht="136" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B58" s="1">
         <v>2026</v>
@@ -1994,21 +1994,21 @@
         <v>2026</v>
       </c>
       <c r="D58" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="F58" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="E58" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="F58" s="1" t="s">
-        <v>148</v>
-      </c>
       <c r="G58" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="59" spans="1:9" ht="136" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B59" s="1">
         <v>2026</v>
@@ -2017,21 +2017,21 @@
         <v>2026</v>
       </c>
       <c r="D59" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="F59" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="E59" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="F59" s="1" t="s">
+      <c r="G59" s="1" t="s">
         <v>142</v>
-      </c>
-      <c r="G59" s="1" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="60" spans="1:9" ht="119" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B60" s="1">
         <v>2025</v>
@@ -2040,21 +2040,21 @@
         <v>2025</v>
       </c>
       <c r="D60" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="F60" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="E60" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="F60" s="1" t="s">
+      <c r="G60" s="1" t="s">
         <v>123</v>
-      </c>
-      <c r="G60" s="1" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="61" spans="1:9" ht="102" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B61" s="1">
         <v>2025</v>
@@ -2063,21 +2063,21 @@
         <v>2025</v>
       </c>
       <c r="D61" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="F61" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="G61" s="1" t="s">
         <v>126</v>
-      </c>
-      <c r="E61" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="F61" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="G61" s="1" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="62" spans="1:9" ht="119" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B62" s="1">
         <v>2025</v>
@@ -2086,21 +2086,21 @@
         <v>2026</v>
       </c>
       <c r="D62" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="E62" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="G62" s="1" t="s">
         <v>144</v>
-      </c>
-      <c r="E62" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="F62" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="G62" s="1" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="63" spans="1:9" ht="102" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B63" s="1">
         <v>2025</v>
@@ -2109,21 +2109,21 @@
         <v>2025</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="64" spans="1:9" ht="85" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B64" s="1">
         <v>2024</v>
@@ -2132,21 +2132,21 @@
         <v>2024</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G64" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="136" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B65" s="1">
         <v>2024</v>
@@ -2155,16 +2155,16 @@
         <v>2024</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F65" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="G65" s="1" t="s">
         <v>133</v>
-      </c>
-      <c r="G65" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated dashboard link for Yakama
</commit_message>
<xml_diff>
--- a/data/cv_entries.xlsx
+++ b/data/cv_entries.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jimwright/Desktop/Resume/wright_cv/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43C0DF74-37BF-384E-9A16-5AAB65BA7E7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D81966F9-120B-B140-8E61-B193AB8C8E2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16180" xr2:uid="{C4D43CE4-6AA2-144D-A346-CE8B2E756935}"/>
   </bookViews>
@@ -490,9 +490,6 @@
     <t>https://jim-asr.shinyapps.io/CommPathLandscape/</t>
   </si>
   <si>
-    <t>https://jim-asr.shinyapps.io/YNHA_Survey_Analysis/</t>
-  </si>
-  <si>
     <t>https://jim-asr.shinyapps.io/F5Siskiyou_DPIL_SurveyResults/</t>
   </si>
   <si>
@@ -533,6 +530,9 @@
   </si>
   <si>
     <t>Developed dashboad in partnership with United Way California Capital Region to help identify opportunities to strengthen outcomes for children, youth, and families through data-informed partnerships with local schools, school districts, and counties.</t>
+  </si>
+  <si>
+    <t>https://asr-ynha-survey-analysis.share.connect.posit.cloud/</t>
   </si>
 </sst>
 </file>
@@ -1765,7 +1765,7 @@
         <v>73</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I47" s="1" t="s">
         <v>96</v>
@@ -1920,16 +1920,16 @@
         <v>2026</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>110</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="55" spans="1:9" ht="204" x14ac:dyDescent="0.2">
@@ -1943,16 +1943,16 @@
         <v>2026</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E55" s="1" t="s">
         <v>110</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="56" spans="1:9" ht="68" x14ac:dyDescent="0.2">
@@ -1966,16 +1966,16 @@
         <v>2026</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>110</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="57" spans="1:9" ht="68" x14ac:dyDescent="0.2">
@@ -1989,16 +1989,16 @@
         <v>2026</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>110</v>
       </c>
       <c r="F57" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="G57" s="1" t="s">
         <v>154</v>
-      </c>
-      <c r="G57" s="1" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="58" spans="1:9" ht="119" x14ac:dyDescent="0.2">
@@ -2021,7 +2021,7 @@
         <v>127</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="59" spans="1:9" ht="68" x14ac:dyDescent="0.2">
@@ -2044,7 +2044,7 @@
         <v>149</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
     </row>
     <row r="60" spans="1:9" ht="136" x14ac:dyDescent="0.2">

</xml_diff>